<commit_message>
Repair accounting portfolio presentation
</commit_message>
<xml_diff>
--- a/accounts-receivable/ar-aging-dashboard/AR_Aging_Dashboard_2026-06-30.xlsx
+++ b/accounts-receivable/ar-aging-dashboard/AR_Aging_Dashboard_2026-06-30.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Data" sheetId="1" r:id="R67de9bb595af4824"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rb9182d19147f4865"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice Detail" sheetId="3" r:id="R512abcf0e4124fcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer Summary" sheetId="4" r:id="R60688d896e694a20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Checks" sheetId="5" r:id="R28ce11eabe9f46ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Data" sheetId="1" r:id="R2cae2b96a38a4c33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R6e42ef89be35427e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice Detail" sheetId="3" r:id="Rf80c6786a55d4cf0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer Summary" sheetId="4" r:id="Racb1fb1ef80642ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Checks" sheetId="5" r:id="R9aec950127674e14"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2856,7 +2856,7 @@
         <x:color rgb="FFC63D3D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4E5"/>
         </x:patternFill>
       </x:fill>
@@ -2867,7 +2867,7 @@
         <x:color rgb="FFC63D3D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCECEC"/>
         </x:patternFill>
       </x:fill>
@@ -2878,7 +2878,7 @@
         <x:color rgb="FFC63D3D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCECEC"/>
         </x:patternFill>
       </x:fill>
@@ -2889,7 +2889,7 @@
         <x:color rgb="FF9A5A00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4E5"/>
         </x:patternFill>
       </x:fill>
@@ -2900,7 +2900,7 @@
         <x:color rgb="FFC63D3D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCECEC"/>
         </x:patternFill>
       </x:fill>
@@ -2911,7 +2911,7 @@
         <x:color rgb="FF6B5CA5"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF1EEFA"/>
         </x:patternFill>
       </x:fill>
@@ -2922,7 +2922,7 @@
         <x:color rgb="FF7A4A00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4E5"/>
         </x:patternFill>
       </x:fill>
@@ -2933,7 +2933,7 @@
         <x:color rgb="FFC63D3D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCECEC"/>
         </x:patternFill>
       </x:fill>
@@ -2944,7 +2944,7 @@
         <x:color rgb="FFC63D3D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCECEC"/>
         </x:patternFill>
       </x:fill>
@@ -2955,7 +2955,7 @@
         <x:color rgb="FF9A5A00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4E5"/>
         </x:patternFill>
       </x:fill>
@@ -2966,7 +2966,7 @@
         <x:color rgb="FFC63D3D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCECEC"/>
         </x:patternFill>
       </x:fill>
@@ -2977,7 +2977,7 @@
         <x:color rgb="FF9A5A00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4E5"/>
         </x:patternFill>
       </x:fill>
@@ -2988,7 +2988,7 @@
         <x:color rgb="FF6B5CA5"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF1EEFA"/>
         </x:patternFill>
       </x:fill>
@@ -2999,7 +2999,7 @@
         <x:color rgb="FF2E7D32"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF5EA"/>
         </x:patternFill>
       </x:fill>
@@ -3010,7 +3010,7 @@
         <x:color rgb="FFC63D3D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCECEC"/>
         </x:patternFill>
       </x:fill>
@@ -3335,7 +3335,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R279df7bb425b4ba3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R24f8eddca07b42bb"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3365,7 +3365,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd4283d2824ff4070"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8e5049e4943d44c4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -4410,7 +4410,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fa201843024432c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R449fbcdd46af4fa7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4593,7 +4593,7 @@
         <x:v>Portfolio owner</x:v>
       </x:c>
       <x:c r="G4" s="80" t="str">
-        <x:v>SanDAce07</x:v>
+        <x:v>Sandesh Lama Tamang</x:v>
       </x:c>
       <x:c r="H4" s="80"/>
       <x:c r="I4" s="82" t="str">
@@ -5209,8 +5209,8 @@
     <x:mergeCell ref="J36:O39"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reff5962692e6405d"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35aba529cb8b43c8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5fe298b7e174d6f"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47b3d950c5434122"/>
 </x:worksheet>
 </file>
 
@@ -7704,7 +7704,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad6d9ac8c310479d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94ea0a62fc4e4d66"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8946,7 +8946,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5865acaaaf394f87"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebb4de7e5a03415f"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">

</xml_diff>